<commit_message>
fix: validate merged GF_X runtime contracts
</commit_message>
<xml_diff>
--- a/GameData/DataTables/Business/ResourceConfig.xlsx
+++ b/GameData/DataTables/Business/ResourceConfig.xlsx
@@ -8,9 +8,55 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet 1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
+</file>
+
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+  <si>
+    <t>#</t>
+  </si>
+  <si>
+    <t>Business table migrated from LegacyProjectArchive/Assets/Resources/DataTable/ResourceConfig.json. GF_X Id is numeric; original business keys are preserved as data columns.</t>
+  </si>
+  <si>
+    <t>Id</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>Name</t>
+  </si>
+  <si>
+    <t>Type</t>
+  </si>
+  <si>
+    <t>LoadPath</t>
+  </si>
+  <si>
+    <t>int</t>
+  </si>
+  <si>
+    <t>string</t>
+  </si>
+  <si>
+    <t>GF_X numeric row id. Original business key is preserved as a data column when its name is not Id.</t>
+  </si>
+  <si>
+    <t>Note</t>
+  </si>
+  <si>
+    <t>资源标识名</t>
+  </si>
+  <si>
+    <t>资源类型，对应 Resources 下子目录名</t>
+  </si>
+  <si>
+    <t>相对 Resources/{Type}/ 的加载路径，不含扩展名</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -18,13 +64,13 @@
   <numFmts count="0"/>
   <fonts count="1">
     <font>
+      <sz val="11"/>
       <name val="Calibri"/>
-      <sz val="11"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -43,7 +89,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -412,106 +458,75 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Business table migrated from LegacyProjectArchive/Assets/Resources/DataTable/ResourceConfig.json. GF_X Id is numeric; original business keys are preserved as data columns.</t>
-        </is>
+      <c r="A1" s="0" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="0" t="s">
+        <v>1</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Id</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Name</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Type</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>LoadPath</t>
-        </is>
+      <c r="A2" s="0" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="0" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="D2" s="0" t="s">
+        <v>4</v>
+      </c>
+      <c r="E2" s="0" t="s">
+        <v>5</v>
+      </c>
+      <c r="F2" s="0" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>int</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
+      <c r="A3" s="0" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="0" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="D3" s="0" t="s">
+        <v>8</v>
+      </c>
+      <c r="E3" s="0" t="s">
+        <v>8</v>
+      </c>
+      <c r="F3" s="0" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>GF_X numeric row id. Original business key is preserved as a data column when its name is not Id.</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Note</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>资源标识名</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>资源类型，对应 Resources 下子目录名</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>相对 Resources/{Type}/ 的加载路径，不含扩展名</t>
-        </is>
+      <c r="A4" s="0" t="s">
+        <v>0</v>
+      </c>
+      <c r="B4" s="0" t="s">
+        <v>9</v>
+      </c>
+      <c r="C4" s="0" t="s">
+        <v>10</v>
+      </c>
+      <c r="D4" s="0" t="s">
+        <v>11</v>
+      </c>
+      <c r="E4" s="0" t="s">
+        <v>12</v>
+      </c>
+      <c r="F4" s="0" t="s">
+        <v>13</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>